<commit_message>
set data type to text
</commit_message>
<xml_diff>
--- a/tests/data/import/xlsx/sample_sentence/doc1.xlsx
+++ b/tests/data/import/xlsx/sample_sentence/doc1.xlsx
@@ -150,8 +150,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -181,88 +185,89 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="10.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="10.58"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="3" style="1" width="10.78"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2"/>
+      <c r="B5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2"/>
+      <c r="B6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="2"/>
+      <c r="B8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="2"/>
+      <c r="B9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="2"/>
+      <c r="B10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="2"/>
+      <c r="B11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="2"/>
+      <c r="B12" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -285,7 +290,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="10.58"/>
   </cols>

</xml_diff>